<commit_message>
fix: remove unsupported vendor chart extensions from gradebook sample
</commit_message>
<xml_diff>
--- a/assets/showcase/gradebook.xlsx
+++ b/assets/showcase/gradebook.xlsx
@@ -1354,13 +1354,6 @@
             <c:showPercent val="0"/>
             <c:showBubbleSize val="1"/>
             <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
-                <c15:showLeaderLines val="0"/>
-                <c15:leaderLines/>
-              </c:ext>
-            </c:extLst>
           </c:dLbls>
           <c:cat>
             <c:strRef>
@@ -1545,11 +1538,6 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext uri="{0b15fc19-7d7d-44ad-8c2d-2c3a37ce22c3}">
-        <chartProps xmlns="https://web.wps.cn/et/2018/main" chartId="{35c50c0a-128b-4dde-a4e6-ff3b34bde8e6}"/>
-      </c:ext>
-    </c:extLst>
   </c:chart>
   <c:txPr>
     <a:bodyPr/>

</xml_diff>

<commit_message>
fix: sanitize xlsx gradebook sample chart extensions for clean baseline validate (#46)
* test: capture gradebook baseline chart validation expectations

* fix: remove unsupported vendor chart extensions from gradebook sample
</commit_message>
<xml_diff>
--- a/assets/showcase/gradebook.xlsx
+++ b/assets/showcase/gradebook.xlsx
@@ -1354,13 +1354,6 @@
             <c:showPercent val="0"/>
             <c:showBubbleSize val="1"/>
             <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
-                <c15:showLeaderLines val="0"/>
-                <c15:leaderLines/>
-              </c:ext>
-            </c:extLst>
           </c:dLbls>
           <c:cat>
             <c:strRef>
@@ -1545,11 +1538,6 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext uri="{0b15fc19-7d7d-44ad-8c2d-2c3a37ce22c3}">
-        <chartProps xmlns="https://web.wps.cn/et/2018/main" chartId="{35c50c0a-128b-4dde-a4e6-ff3b34bde8e6}"/>
-      </c:ext>
-    </c:extLst>
   </c:chart>
   <c:txPr>
     <a:bodyPr/>

</xml_diff>